<commit_message>
sales_model: godkendte beskrivelser skrevet til TMDL
- 107 godkendte beskrivelser skrevet tilbage som ///-linjer i alle 13
  tabelfiler. Ingen DAX, M eller egenskaber er ændret.
- Kataloget er genereret igen: alle 107 beskrivelser står som Godkendt,
  og en ny tørkørsel af tilbageskrivningen giver 0 ændringer.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013At67Gwi9xCc2C5qN1Bh34
</commit_message>
<xml_diff>
--- a/output/sales_model/docs/catalog.xlsx
+++ b/output/sales_model/docs/catalog.xlsx
@@ -488,7 +488,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-29 20:02</t>
+          <t>2026-10-29 20:03</t>
         </is>
       </c>
     </row>
@@ -577,7 +577,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>107</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -607,7 +607,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0</v>
+        <v>107</v>
       </c>
     </row>
     <row r="16">
@@ -826,12 +826,12 @@
       <c r="O2" s="4" t="inlineStr"/>
       <c r="P2" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -889,12 +889,12 @@
       <c r="O3" s="4" t="inlineStr"/>
       <c r="P3" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -952,12 +952,12 @@
       <c r="O4" s="4" t="inlineStr"/>
       <c r="P4" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -1003,12 +1003,12 @@
       <c r="O5" s="4" t="inlineStr"/>
       <c r="P5" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -1066,12 +1066,12 @@
       <c r="O6" s="4" t="inlineStr"/>
       <c r="P6" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -1125,12 +1125,12 @@
       <c r="O7" s="4" t="inlineStr"/>
       <c r="P7" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -1188,12 +1188,12 @@
       <c r="O8" s="4" t="inlineStr"/>
       <c r="P8" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -1251,12 +1251,12 @@
       <c r="O9" s="4" t="inlineStr"/>
       <c r="P9" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -1314,12 +1314,12 @@
       <c r="O10" s="4" t="inlineStr"/>
       <c r="P10" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -1377,12 +1377,12 @@
       <c r="O11" s="4" t="inlineStr"/>
       <c r="P11" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -1440,12 +1440,12 @@
       <c r="O12" s="4" t="inlineStr"/>
       <c r="P12" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -1503,12 +1503,12 @@
       <c r="O13" s="4" t="inlineStr"/>
       <c r="P13" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -1570,12 +1570,12 @@
       <c r="O14" s="4" t="inlineStr"/>
       <c r="P14" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -1794,12 +1794,12 @@
       <c r="T2" s="4" t="inlineStr"/>
       <c r="U2" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -1862,12 +1862,12 @@
       <c r="T3" s="4" t="inlineStr"/>
       <c r="U3" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -1934,12 +1934,12 @@
       <c r="T4" s="4" t="inlineStr"/>
       <c r="U4" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -2006,12 +2006,12 @@
       <c r="T5" s="4" t="inlineStr"/>
       <c r="U5" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -2070,12 +2070,12 @@
       <c r="T6" s="4" t="inlineStr"/>
       <c r="U6" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -2138,12 +2138,12 @@
       <c r="T7" s="4" t="inlineStr"/>
       <c r="U7" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -2206,12 +2206,12 @@
       <c r="T8" s="4" t="inlineStr"/>
       <c r="U8" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -2278,12 +2278,12 @@
       <c r="T9" s="4" t="inlineStr"/>
       <c r="U9" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -2346,12 +2346,12 @@
       <c r="T10" s="4" t="inlineStr"/>
       <c r="U10" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -2410,12 +2410,12 @@
       <c r="T11" s="4" t="inlineStr"/>
       <c r="U11" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -2482,12 +2482,12 @@
       <c r="T12" s="4" t="inlineStr"/>
       <c r="U12" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -2550,12 +2550,12 @@
       <c r="T13" s="4" t="inlineStr"/>
       <c r="U13" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -2622,12 +2622,12 @@
       <c r="T14" s="4" t="inlineStr"/>
       <c r="U14" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -2686,12 +2686,12 @@
       <c r="T15" s="4" t="inlineStr"/>
       <c r="U15" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -2758,12 +2758,12 @@
       <c r="T16" s="4" t="inlineStr"/>
       <c r="U16" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -2822,12 +2822,12 @@
       <c r="T17" s="4" t="inlineStr"/>
       <c r="U17" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -2890,12 +2890,12 @@
       <c r="T18" s="4" t="inlineStr"/>
       <c r="U18" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -2954,12 +2954,12 @@
       <c r="T19" s="4" t="inlineStr"/>
       <c r="U19" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -3026,12 +3026,12 @@
       <c r="T20" s="4" t="inlineStr"/>
       <c r="U20" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -3090,12 +3090,12 @@
       <c r="T21" s="4" t="inlineStr"/>
       <c r="U21" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -3154,12 +3154,12 @@
       <c r="T22" s="4" t="inlineStr"/>
       <c r="U22" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -3218,12 +3218,12 @@
       <c r="T23" s="4" t="inlineStr"/>
       <c r="U23" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -3282,12 +3282,12 @@
       <c r="T24" s="4" t="inlineStr"/>
       <c r="U24" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V24" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -3342,12 +3342,12 @@
       <c r="T25" s="4" t="inlineStr"/>
       <c r="U25" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V25" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -3410,12 +3410,12 @@
       <c r="T26" s="4" t="inlineStr"/>
       <c r="U26" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V26" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -3478,12 +3478,12 @@
       <c r="T27" s="4" t="inlineStr"/>
       <c r="U27" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V27" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -3538,12 +3538,12 @@
       <c r="T28" s="4" t="inlineStr"/>
       <c r="U28" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V28" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -3602,12 +3602,12 @@
       <c r="T29" s="4" t="inlineStr"/>
       <c r="U29" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V29" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -3666,12 +3666,12 @@
       <c r="T30" s="4" t="inlineStr"/>
       <c r="U30" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V30" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -3738,12 +3738,12 @@
       <c r="T31" s="4" t="inlineStr"/>
       <c r="U31" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V31" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -3802,12 +3802,12 @@
       <c r="T32" s="4" t="inlineStr"/>
       <c r="U32" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V32" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -3874,12 +3874,12 @@
       <c r="T33" s="4" t="inlineStr"/>
       <c r="U33" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V33" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -3938,12 +3938,12 @@
       <c r="T34" s="4" t="inlineStr"/>
       <c r="U34" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V34" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -3998,12 +3998,12 @@
       <c r="T35" s="4" t="inlineStr"/>
       <c r="U35" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V35" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -4058,12 +4058,12 @@
       <c r="T36" s="4" t="inlineStr"/>
       <c r="U36" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V36" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -4126,12 +4126,12 @@
       <c r="T37" s="4" t="inlineStr"/>
       <c r="U37" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V37" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -4190,12 +4190,12 @@
       <c r="T38" s="4" t="inlineStr"/>
       <c r="U38" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V38" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -4262,12 +4262,12 @@
       <c r="T39" s="4" t="inlineStr"/>
       <c r="U39" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V39" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -4334,12 +4334,12 @@
       <c r="T40" s="4" t="inlineStr"/>
       <c r="U40" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V40" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -4406,12 +4406,12 @@
       <c r="T41" s="4" t="inlineStr"/>
       <c r="U41" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V41" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -4474,12 +4474,12 @@
       <c r="T42" s="4" t="inlineStr"/>
       <c r="U42" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V42" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -4546,12 +4546,12 @@
       <c r="T43" s="4" t="inlineStr"/>
       <c r="U43" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V43" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -4618,12 +4618,12 @@
       <c r="T44" s="4" t="inlineStr"/>
       <c r="U44" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V44" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -4690,12 +4690,12 @@
       <c r="T45" s="4" t="inlineStr"/>
       <c r="U45" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V45" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -4758,12 +4758,12 @@
       <c r="T46" s="4" t="inlineStr"/>
       <c r="U46" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V46" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -4826,12 +4826,12 @@
       <c r="T47" s="4" t="inlineStr"/>
       <c r="U47" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V47" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -4898,12 +4898,12 @@
       <c r="T48" s="4" t="inlineStr"/>
       <c r="U48" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V48" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -4962,12 +4962,12 @@
       <c r="T49" s="4" t="inlineStr"/>
       <c r="U49" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V49" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -5026,12 +5026,12 @@
       <c r="T50" s="4" t="inlineStr"/>
       <c r="U50" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V50" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -5098,12 +5098,12 @@
       <c r="T51" s="4" t="inlineStr"/>
       <c r="U51" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V51" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -5166,12 +5166,12 @@
       <c r="T52" s="4" t="inlineStr"/>
       <c r="U52" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V52" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -5234,12 +5234,12 @@
       <c r="T53" s="4" t="inlineStr"/>
       <c r="U53" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V53" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -5302,12 +5302,12 @@
       <c r="T54" s="4" t="inlineStr"/>
       <c r="U54" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V54" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -5370,12 +5370,12 @@
       <c r="T55" s="4" t="inlineStr"/>
       <c r="U55" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V55" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -5434,12 +5434,12 @@
       <c r="T56" s="4" t="inlineStr"/>
       <c r="U56" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V56" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -5498,12 +5498,12 @@
       <c r="T57" s="4" t="inlineStr"/>
       <c r="U57" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V57" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -5570,12 +5570,12 @@
       <c r="T58" s="4" t="inlineStr"/>
       <c r="U58" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V58" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -5642,12 +5642,12 @@
       <c r="T59" s="4" t="inlineStr"/>
       <c r="U59" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V59" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -5714,12 +5714,12 @@
       <c r="T60" s="4" t="inlineStr"/>
       <c r="U60" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V60" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -5782,12 +5782,12 @@
       <c r="T61" s="4" t="inlineStr"/>
       <c r="U61" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V61" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -5850,12 +5850,12 @@
       <c r="T62" s="4" t="inlineStr"/>
       <c r="U62" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V62" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -5918,12 +5918,12 @@
       <c r="T63" s="4" t="inlineStr"/>
       <c r="U63" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V63" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -5986,12 +5986,12 @@
       <c r="T64" s="4" t="inlineStr"/>
       <c r="U64" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V64" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -6054,12 +6054,12 @@
       <c r="T65" s="4" t="inlineStr"/>
       <c r="U65" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V65" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -6126,12 +6126,12 @@
       <c r="T66" s="4" t="inlineStr"/>
       <c r="U66" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V66" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -6202,12 +6202,12 @@
       <c r="T67" s="4" t="inlineStr"/>
       <c r="U67" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V67" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -6270,12 +6270,12 @@
       <c r="T68" s="4" t="inlineStr"/>
       <c r="U68" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V68" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -6484,12 +6484,12 @@
       <c r="R2" s="4" t="inlineStr"/>
       <c r="S2" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -6554,12 +6554,12 @@
       <c r="R3" s="4" t="inlineStr"/>
       <c r="S3" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -6624,12 +6624,12 @@
       <c r="R4" s="4" t="inlineStr"/>
       <c r="S4" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -6690,12 +6690,12 @@
       <c r="R5" s="4" t="inlineStr"/>
       <c r="S5" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -6760,12 +6760,12 @@
       <c r="R6" s="4" t="inlineStr"/>
       <c r="S6" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -6818,12 +6818,12 @@
       <c r="R7" s="4" t="inlineStr"/>
       <c r="S7" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -6884,12 +6884,12 @@
       <c r="R8" s="4" t="inlineStr"/>
       <c r="S8" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -6950,12 +6950,12 @@
       <c r="R9" s="4" t="inlineStr"/>
       <c r="S9" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -7020,12 +7020,12 @@
       <c r="R10" s="4" t="inlineStr"/>
       <c r="S10" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -7090,12 +7090,12 @@
       <c r="R11" s="4" t="inlineStr"/>
       <c r="S11" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -7160,12 +7160,12 @@
       <c r="R12" s="4" t="inlineStr"/>
       <c r="S12" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -7226,12 +7226,12 @@
       <c r="R13" s="4" t="inlineStr"/>
       <c r="S13" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -7296,12 +7296,12 @@
       <c r="R14" s="4" t="inlineStr"/>
       <c r="S14" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -7362,12 +7362,12 @@
       <c r="R15" s="4" t="inlineStr"/>
       <c r="S15" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -7428,12 +7428,12 @@
       <c r="R16" s="4" t="inlineStr"/>
       <c r="S16" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -7498,12 +7498,12 @@
       <c r="R17" s="4" t="inlineStr"/>
       <c r="S17" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -7572,12 +7572,12 @@
       <c r="R18" s="4" t="inlineStr"/>
       <c r="S18" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -7638,12 +7638,12 @@
       <c r="R19" s="4" t="inlineStr"/>
       <c r="S19" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -7708,12 +7708,12 @@
       <c r="R20" s="4" t="inlineStr"/>
       <c r="S20" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -7778,12 +7778,12 @@
       <c r="R21" s="4" t="inlineStr"/>
       <c r="S21" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -7844,12 +7844,12 @@
       <c r="R22" s="4" t="inlineStr"/>
       <c r="S22" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -7914,12 +7914,12 @@
       <c r="R23" s="4" t="inlineStr"/>
       <c r="S23" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -7984,12 +7984,12 @@
       <c r="R24" s="4" t="inlineStr"/>
       <c r="S24" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -8050,12 +8050,12 @@
       <c r="R25" s="4" t="inlineStr"/>
       <c r="S25" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -8116,12 +8116,12 @@
       <c r="R26" s="4" t="inlineStr"/>
       <c r="S26" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -8186,12 +8186,12 @@
       <c r="R27" s="4" t="inlineStr"/>
       <c r="S27" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>
@@ -8252,12 +8252,12 @@
       <c r="R28" s="4" t="inlineStr"/>
       <c r="S28" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Excel</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
sales_model: Opstrøms kilde udfyldt og rettet lineage for kategori og lager
- catalog.xlsx: "Opstrøms kilde" er udfyldt for alle 13 tabeller og
  67 kolonner med sti, ark og kolonne i data/silver/Silver_Excel.xlsx.
  Genererede felter (surrogatnøgler, dim_date, dim_channel og beregnede
  beløb) er beskrevet som sådan.
- Kataloget er genereret igen med den rettede parser (claude-powerbi-skills
  PR #2): dim_product[category] og [subcategory] når nu ud til
  subcategories › CategorySubcategory, og fact_inventory[stock_qty] viser
  unpivot af månedskolonnerne.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013At67Gwi9xCc2C5qN1Bh34
</commit_message>
<xml_diff>
--- a/output/sales_model/docs/catalog.xlsx
+++ b/output/sales_model/docs/catalog.xlsx
@@ -488,7 +488,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-29 20:03</t>
+          <t>2026-10-29 20:08</t>
         </is>
       </c>
     </row>
@@ -696,7 +696,7 @@
     <col width="60" customWidth="1" min="12" max="12"/>
     <col width="10" customWidth="1" min="13" max="13"/>
     <col width="11" customWidth="1" min="14" max="14"/>
-    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="45" customWidth="1" min="15" max="15"/>
     <col width="10" customWidth="1" min="16" max="16"/>
     <col width="19" customWidth="1" min="17" max="17"/>
   </cols>
@@ -823,7 +823,11 @@
       </c>
       <c r="M2" s="4" t="inlineStr"/>
       <c r="N2" s="4" t="inlineStr"/>
-      <c r="O2" s="4" t="inlineStr"/>
+      <c r="O2" s="4" t="inlineStr">
+        <is>
+          <t>Ingen – measure-tabel i Power BI</t>
+        </is>
+      </c>
       <c r="P2" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -886,7 +890,11 @@
       </c>
       <c r="M3" s="4" t="inlineStr"/>
       <c r="N3" s="4" t="inlineStr"/>
-      <c r="O3" s="4" t="inlineStr"/>
+      <c r="O3" s="4" t="inlineStr">
+        <is>
+          <t>data/silver/Silver_Excel.xlsx › campaign_skus (CampaignName, PromotedSKUs) matchet mod dim_campaign og dim_product</t>
+        </is>
+      </c>
       <c r="P3" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -949,7 +957,11 @@
       </c>
       <c r="M4" s="4" t="inlineStr"/>
       <c r="N4" s="4" t="inlineStr"/>
-      <c r="O4" s="4" t="inlineStr"/>
+      <c r="O4" s="4" t="inlineStr">
+        <is>
+          <t>data/silver/Silver_Excel.xlsx › CAMPAIGN_LOG</t>
+        </is>
+      </c>
       <c r="P4" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -1000,7 +1012,11 @@
       </c>
       <c r="M5" s="4" t="inlineStr"/>
       <c r="N5" s="4" t="inlineStr"/>
-      <c r="O5" s="4" t="inlineStr"/>
+      <c r="O5" s="4" t="inlineStr">
+        <is>
+          <t>Fast liste i Power Query – ingen kilde i silver</t>
+        </is>
+      </c>
       <c r="P5" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -1063,7 +1079,11 @@
       </c>
       <c r="M6" s="4" t="inlineStr"/>
       <c r="N6" s="4" t="inlineStr"/>
-      <c r="O6" s="4" t="inlineStr"/>
+      <c r="O6" s="4" t="inlineStr">
+        <is>
+          <t>data/silver/Silver_Excel.xlsx › Address, CUST_MASTER, cities, customer_contacts, user_details</t>
+        </is>
+      </c>
       <c r="P6" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -1122,7 +1142,11 @@
       </c>
       <c r="M7" s="4" t="inlineStr"/>
       <c r="N7" s="4" t="inlineStr"/>
-      <c r="O7" s="4" t="inlineStr"/>
+      <c r="O7" s="4" t="inlineStr">
+        <is>
+          <t>Genereres i Power Query ud fra datoerne i ordrer, kampagner, lager og salgsmål</t>
+        </is>
+      </c>
       <c r="P7" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -1159,7 +1183,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>products (Sheet)</t>
+          <t>products (Sheet), subcategories (Sheet)</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1185,7 +1209,11 @@
       </c>
       <c r="M8" s="4" t="inlineStr"/>
       <c r="N8" s="4" t="inlineStr"/>
-      <c r="O8" s="4" t="inlineStr"/>
+      <c r="O8" s="4" t="inlineStr">
+        <is>
+          <t>data/silver/Silver_Excel.xlsx › products, subcategories</t>
+        </is>
+      </c>
       <c r="P8" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -1248,7 +1276,11 @@
       </c>
       <c r="M9" s="4" t="inlineStr"/>
       <c r="N9" s="4" t="inlineStr"/>
-      <c r="O9" s="4" t="inlineStr"/>
+      <c r="O9" s="4" t="inlineStr">
+        <is>
+          <t>data/silver/Silver_Excel.xlsx › cities</t>
+        </is>
+      </c>
       <c r="P9" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -1311,7 +1343,11 @@
       </c>
       <c r="M10" s="4" t="inlineStr"/>
       <c r="N10" s="4" t="inlineStr"/>
-      <c r="O10" s="4" t="inlineStr"/>
+      <c r="O10" s="4" t="inlineStr">
+        <is>
+          <t>data/silver/Silver_Excel.xlsx › CAMPAIGN_LOG</t>
+        </is>
+      </c>
       <c r="P10" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -1374,7 +1410,11 @@
       </c>
       <c r="M11" s="4" t="inlineStr"/>
       <c r="N11" s="4" t="inlineStr"/>
-      <c r="O11" s="4" t="inlineStr"/>
+      <c r="O11" s="4" t="inlineStr">
+        <is>
+          <t>data/silver/Silver_Excel.xlsx › inventory</t>
+        </is>
+      </c>
       <c r="P11" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -1437,7 +1477,11 @@
       </c>
       <c r="M12" s="4" t="inlineStr"/>
       <c r="N12" s="4" t="inlineStr"/>
-      <c r="O12" s="4" t="inlineStr"/>
+      <c r="O12" s="4" t="inlineStr">
+        <is>
+          <t>data/silver/Silver_Excel.xlsx › ORDERS_2025 + ORDERS_2026 (ordrehoved) og order_line_items (linjer)</t>
+        </is>
+      </c>
       <c r="P12" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -1500,7 +1544,11 @@
       </c>
       <c r="M13" s="4" t="inlineStr"/>
       <c r="N13" s="4" t="inlineStr"/>
-      <c r="O13" s="4" t="inlineStr"/>
+      <c r="O13" s="4" t="inlineStr">
+        <is>
+          <t>data/silver/Silver_Excel.xlsx › sales_targets</t>
+        </is>
+      </c>
       <c r="P13" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -1567,7 +1615,11 @@
       </c>
       <c r="M14" s="4" t="inlineStr"/>
       <c r="N14" s="4" t="inlineStr"/>
-      <c r="O14" s="4" t="inlineStr"/>
+      <c r="O14" s="4" t="inlineStr">
+        <is>
+          <t>data/silver/Silver_Excel.xlsx › security</t>
+        </is>
+      </c>
       <c r="P14" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -1608,7 +1660,7 @@
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="42" customWidth="1" min="10" max="10"/>
+    <col width="45" customWidth="1" min="10" max="10"/>
     <col width="45" customWidth="1" min="11" max="11"/>
     <col width="60" customWidth="1" min="12" max="12"/>
     <col width="60" customWidth="1" min="13" max="13"/>
@@ -1618,7 +1670,7 @@
     <col width="60" customWidth="1" min="17" max="17"/>
     <col width="10" customWidth="1" min="18" max="18"/>
     <col width="18" customWidth="1" min="19" max="19"/>
-    <col width="16" customWidth="1" min="20" max="20"/>
+    <col width="45" customWidth="1" min="20" max="20"/>
     <col width="10" customWidth="1" min="21" max="21"/>
     <col width="19" customWidth="1" min="22" max="22"/>
   </cols>
@@ -1791,7 +1843,11 @@
       </c>
       <c r="R2" s="4" t="inlineStr"/>
       <c r="S2" s="4" t="inlineStr"/>
-      <c r="T2" s="4" t="inlineStr"/>
+      <c r="T2" s="4" t="inlineStr">
+        <is>
+          <t>Opslag af dim_campaign[campaign_key] (surrogatnøgle genereret i Power Query)</t>
+        </is>
+      </c>
       <c r="U2" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -1859,7 +1915,11 @@
       </c>
       <c r="R3" s="4" t="inlineStr"/>
       <c r="S3" s="4" t="inlineStr"/>
-      <c r="T3" s="4" t="inlineStr"/>
+      <c r="T3" s="4" t="inlineStr">
+        <is>
+          <t>Opslag af dim_product[product_key] (surrogatnøgle genereret i Power Query)</t>
+        </is>
+      </c>
       <c r="U3" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -1931,7 +1991,11 @@
       </c>
       <c r="R4" s="4" t="inlineStr"/>
       <c r="S4" s="4" t="inlineStr"/>
-      <c r="T4" s="4" t="inlineStr"/>
+      <c r="T4" s="4" t="inlineStr">
+        <is>
+          <t>Surrogatnøgle genereret i Power Query (fortløbende, -1 = Ukendt)</t>
+        </is>
+      </c>
       <c r="U4" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -2003,7 +2067,11 @@
           <t>Mulig PII - vurdér</t>
         </is>
       </c>
-      <c r="T5" s="4" t="inlineStr"/>
+      <c r="T5" s="4" t="inlineStr">
+        <is>
+          <t>data/silver/Silver_Excel.xlsx › CAMPAIGN_LOG › CampaignName</t>
+        </is>
+      </c>
       <c r="U5" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -2067,7 +2135,11 @@
       </c>
       <c r="R6" s="4" t="inlineStr"/>
       <c r="S6" s="4" t="inlineStr"/>
-      <c r="T6" s="4" t="inlineStr"/>
+      <c r="T6" s="4" t="inlineStr">
+        <is>
+          <t>data/silver/Silver_Excel.xlsx › CAMPAIGN_LOG › Channel</t>
+        </is>
+      </c>
       <c r="U6" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -2135,7 +2207,11 @@
       </c>
       <c r="R7" s="4" t="inlineStr"/>
       <c r="S7" s="4" t="inlineStr"/>
-      <c r="T7" s="4" t="inlineStr"/>
+      <c r="T7" s="4" t="inlineStr">
+        <is>
+          <t>data/silver/Silver_Excel.xlsx › CAMPAIGN_LOG › StartDate</t>
+        </is>
+      </c>
       <c r="U7" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -2203,7 +2279,11 @@
       </c>
       <c r="R8" s="4" t="inlineStr"/>
       <c r="S8" s="4" t="inlineStr"/>
-      <c r="T8" s="4" t="inlineStr"/>
+      <c r="T8" s="4" t="inlineStr">
+        <is>
+          <t>data/silver/Silver_Excel.xlsx › CAMPAIGN_LOG › EndDate</t>
+        </is>
+      </c>
       <c r="U8" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -2275,7 +2355,11 @@
       </c>
       <c r="R9" s="4" t="inlineStr"/>
       <c r="S9" s="4" t="inlineStr"/>
-      <c r="T9" s="4" t="inlineStr"/>
+      <c r="T9" s="4" t="inlineStr">
+        <is>
+          <t>data/silver/Silver_Excel.xlsx › CAMPAIGN_LOG › Budget</t>
+        </is>
+      </c>
       <c r="U9" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -2343,7 +2427,11 @@
       </c>
       <c r="R10" s="4" t="inlineStr"/>
       <c r="S10" s="4" t="inlineStr"/>
-      <c r="T10" s="4" t="inlineStr"/>
+      <c r="T10" s="4" t="inlineStr">
+        <is>
+          <t>Fast liste i Power Query (dim_channel) – ingen kilde i silver</t>
+        </is>
+      </c>
       <c r="U10" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -2407,7 +2495,11 @@
           <t>Mulig PII - vurdér</t>
         </is>
       </c>
-      <c r="T11" s="4" t="inlineStr"/>
+      <c r="T11" s="4" t="inlineStr">
+        <is>
+          <t>Fast liste i Power Query (dim_channel) – ingen kilde i silver</t>
+        </is>
+      </c>
       <c r="U11" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -2479,7 +2571,11 @@
       </c>
       <c r="R12" s="4" t="inlineStr"/>
       <c r="S12" s="4" t="inlineStr"/>
-      <c r="T12" s="4" t="inlineStr"/>
+      <c r="T12" s="4" t="inlineStr">
+        <is>
+          <t>Surrogatnøgle genereret i Power Query (fortløbende, -1 = Ukendt)</t>
+        </is>
+      </c>
       <c r="U12" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -2547,7 +2643,11 @@
       </c>
       <c r="R13" s="4" t="inlineStr"/>
       <c r="S13" s="4" t="inlineStr"/>
-      <c r="T13" s="4" t="inlineStr"/>
+      <c r="T13" s="4" t="inlineStr">
+        <is>
+          <t>data/silver/Silver_Excel.xlsx › CUST_MASTER › CustomerID</t>
+        </is>
+      </c>
       <c r="U13" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -2619,7 +2719,11 @@
           <t>Mulig PII - vurdér</t>
         </is>
       </c>
-      <c r="T14" s="4" t="inlineStr"/>
+      <c r="T14" s="4" t="inlineStr">
+        <is>
+          <t>data/silver/Silver_Excel.xlsx › CUST_MASTER › CustomerName</t>
+        </is>
+      </c>
       <c r="U14" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -2683,7 +2787,11 @@
       </c>
       <c r="R15" s="4" t="inlineStr"/>
       <c r="S15" s="4" t="inlineStr"/>
-      <c r="T15" s="4" t="inlineStr"/>
+      <c r="T15" s="4" t="inlineStr">
+        <is>
+          <t>data/silver/Silver_Excel.xlsx › CUST_MASTER › Segment</t>
+        </is>
+      </c>
       <c r="U15" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -2755,7 +2863,11 @@
           <t>Mulig PII - vurdér</t>
         </is>
       </c>
-      <c r="T16" s="4" t="inlineStr"/>
+      <c r="T16" s="4" t="inlineStr">
+        <is>
+          <t>data/silver/Silver_Excel.xlsx › CUST_MASTER › AccountManager</t>
+        </is>
+      </c>
       <c r="U16" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -2819,7 +2931,11 @@
       </c>
       <c r="R17" s="4" t="inlineStr"/>
       <c r="S17" s="4" t="inlineStr"/>
-      <c r="T17" s="4" t="inlineStr"/>
+      <c r="T17" s="4" t="inlineStr">
+        <is>
+          <t>data/silver/Silver_Excel.xlsx › CUST_MASTER › PaymentTerms</t>
+        </is>
+      </c>
       <c r="U17" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -2887,7 +3003,11 @@
       </c>
       <c r="R18" s="4" t="inlineStr"/>
       <c r="S18" s="4" t="inlineStr"/>
-      <c r="T18" s="4" t="inlineStr"/>
+      <c r="T18" s="4" t="inlineStr">
+        <is>
+          <t>data/silver/Silver_Excel.xlsx › user_details › CreditLimit</t>
+        </is>
+      </c>
       <c r="U18" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -2951,7 +3071,11 @@
       </c>
       <c r="R19" s="4" t="inlineStr"/>
       <c r="S19" s="4" t="inlineStr"/>
-      <c r="T19" s="4" t="inlineStr"/>
+      <c r="T19" s="4" t="inlineStr">
+        <is>
+          <t>data/silver/Silver_Excel.xlsx › Address › Street</t>
+        </is>
+      </c>
       <c r="U19" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -3023,7 +3147,11 @@
           <t>Mulig PII - vurdér</t>
         </is>
       </c>
-      <c r="T20" s="4" t="inlineStr"/>
+      <c r="T20" s="4" t="inlineStr">
+        <is>
+          <t>data/silver/Silver_Excel.xlsx › Address › CityName</t>
+        </is>
+      </c>
       <c r="U20" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -3087,7 +3215,11 @@
       </c>
       <c r="R21" s="4" t="inlineStr"/>
       <c r="S21" s="4" t="inlineStr"/>
-      <c r="T21" s="4" t="inlineStr"/>
+      <c r="T21" s="4" t="inlineStr">
+        <is>
+          <t>data/silver/Silver_Excel.xlsx › cities › RegionName</t>
+        </is>
+      </c>
       <c r="U21" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -3151,7 +3283,11 @@
       </c>
       <c r="R22" s="4" t="inlineStr"/>
       <c r="S22" s="4" t="inlineStr"/>
-      <c r="T22" s="4" t="inlineStr"/>
+      <c r="T22" s="4" t="inlineStr">
+        <is>
+          <t>data/silver/Silver_Excel.xlsx › customer_contacts › ContactName</t>
+        </is>
+      </c>
       <c r="U22" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -3215,7 +3351,11 @@
       </c>
       <c r="R23" s="4" t="inlineStr"/>
       <c r="S23" s="4" t="inlineStr"/>
-      <c r="T23" s="4" t="inlineStr"/>
+      <c r="T23" s="4" t="inlineStr">
+        <is>
+          <t>Genereres i Power Query (dim_date)</t>
+        </is>
+      </c>
       <c r="U23" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -3279,7 +3419,11 @@
       </c>
       <c r="R24" s="4" t="inlineStr"/>
       <c r="S24" s="4" t="inlineStr"/>
-      <c r="T24" s="4" t="inlineStr"/>
+      <c r="T24" s="4" t="inlineStr">
+        <is>
+          <t>Genereres i Power Query (dim_date)</t>
+        </is>
+      </c>
       <c r="U24" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -3339,7 +3483,11 @@
       </c>
       <c r="R25" s="4" t="inlineStr"/>
       <c r="S25" s="4" t="inlineStr"/>
-      <c r="T25" s="4" t="inlineStr"/>
+      <c r="T25" s="4" t="inlineStr">
+        <is>
+          <t>Genereres i Power Query (dim_date)</t>
+        </is>
+      </c>
       <c r="U25" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -3407,7 +3555,11 @@
       </c>
       <c r="R26" s="4" t="inlineStr"/>
       <c r="S26" s="4" t="inlineStr"/>
-      <c r="T26" s="4" t="inlineStr"/>
+      <c r="T26" s="4" t="inlineStr">
+        <is>
+          <t>Genereres i Power Query (dim_date)</t>
+        </is>
+      </c>
       <c r="U26" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -3475,7 +3627,11 @@
           <t>Mulig PII - vurdér</t>
         </is>
       </c>
-      <c r="T27" s="4" t="inlineStr"/>
+      <c r="T27" s="4" t="inlineStr">
+        <is>
+          <t>Genereres i Power Query (dim_date)</t>
+        </is>
+      </c>
       <c r="U27" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -3535,7 +3691,11 @@
       </c>
       <c r="R28" s="4" t="inlineStr"/>
       <c r="S28" s="4" t="inlineStr"/>
-      <c r="T28" s="4" t="inlineStr"/>
+      <c r="T28" s="4" t="inlineStr">
+        <is>
+          <t>Genereres i Power Query (dim_date)</t>
+        </is>
+      </c>
       <c r="U28" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -3599,7 +3759,11 @@
       </c>
       <c r="R29" s="4" t="inlineStr"/>
       <c r="S29" s="4" t="inlineStr"/>
-      <c r="T29" s="4" t="inlineStr"/>
+      <c r="T29" s="4" t="inlineStr">
+        <is>
+          <t>Genereres i Power Query (dim_date)</t>
+        </is>
+      </c>
       <c r="U29" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -3663,7 +3827,11 @@
       </c>
       <c r="R30" s="4" t="inlineStr"/>
       <c r="S30" s="4" t="inlineStr"/>
-      <c r="T30" s="4" t="inlineStr"/>
+      <c r="T30" s="4" t="inlineStr">
+        <is>
+          <t>Genereres i Power Query (dim_date)</t>
+        </is>
+      </c>
       <c r="U30" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -3735,7 +3903,11 @@
       </c>
       <c r="R31" s="4" t="inlineStr"/>
       <c r="S31" s="4" t="inlineStr"/>
-      <c r="T31" s="4" t="inlineStr"/>
+      <c r="T31" s="4" t="inlineStr">
+        <is>
+          <t>Surrogatnøgle genereret i Power Query (fortløbende, -1 = Ukendt)</t>
+        </is>
+      </c>
       <c r="U31" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -3799,7 +3971,11 @@
       </c>
       <c r="R32" s="4" t="inlineStr"/>
       <c r="S32" s="4" t="inlineStr"/>
-      <c r="T32" s="4" t="inlineStr"/>
+      <c r="T32" s="4" t="inlineStr">
+        <is>
+          <t>data/silver/Silver_Excel.xlsx › products › ProductCode</t>
+        </is>
+      </c>
       <c r="U32" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -3871,7 +4047,11 @@
           <t>Mulig PII - vurdér</t>
         </is>
       </c>
-      <c r="T33" s="4" t="inlineStr"/>
+      <c r="T33" s="4" t="inlineStr">
+        <is>
+          <t>data/silver/Silver_Excel.xlsx › products › ProductName</t>
+        </is>
+      </c>
       <c r="U33" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -3935,7 +4115,11 @@
       </c>
       <c r="R34" s="4" t="inlineStr"/>
       <c r="S34" s="4" t="inlineStr"/>
-      <c r="T34" s="4" t="inlineStr"/>
+      <c r="T34" s="4" t="inlineStr">
+        <is>
+          <t>data/silver/Silver_Excel.xlsx › products › Brand</t>
+        </is>
+      </c>
       <c r="U34" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -3975,13 +4159,17 @@
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr">
         <is>
-          <t>SubLower[Category]</t>
-        </is>
-      </c>
-      <c r="K35" t="inlineStr"/>
+          <t>subcategories (Sheet).CategorySubcategory</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>Excel File: C:\Users\maria\Desktop\Claude\Data Modeling\data\silver\Silver_Excel.xlsx</t>
+        </is>
+      </c>
       <c r="L35" s="5" t="inlineStr">
         <is>
-          <t>dim_product: Hentet via join (SubLower[Category]) → dim_product: Omdøbt (Category → category) → dim_product: Samlet (append) (Typer, Ukendt)</t>
+          <t>slv_subcategory: Navigation (subcategories (Sheet)) → slv_subcategory: Opdelt (CategorySubcategory → Category (skilletegn "|")) → slv_subcategory: Transformeret ({"Category", each Text.Proper(Text.Trim(_)), type text}) → dim_product: Hentet via join (SubLower[Category]) → dim_product: Omdøbt (Category → category) → dim_product: Samlet (append) (Typer, Ukendt)</t>
         </is>
       </c>
       <c r="M35" s="5" t="inlineStr"/>
@@ -3995,7 +4183,11 @@
       </c>
       <c r="R35" s="4" t="inlineStr"/>
       <c r="S35" s="4" t="inlineStr"/>
-      <c r="T35" s="4" t="inlineStr"/>
+      <c r="T35" s="4" t="inlineStr">
+        <is>
+          <t>data/silver/Silver_Excel.xlsx › subcategories › CategorySubcategory (delen før "|"), matchet på underkategori</t>
+        </is>
+      </c>
       <c r="U35" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -4035,13 +4227,17 @@
       <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr">
         <is>
-          <t>SubLower[Subcategory]</t>
-        </is>
-      </c>
-      <c r="K36" t="inlineStr"/>
+          <t>subcategories (Sheet).CategorySubcategory</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>Excel File: C:\Users\maria\Desktop\Claude\Data Modeling\data\silver\Silver_Excel.xlsx</t>
+        </is>
+      </c>
       <c r="L36" s="5" t="inlineStr">
         <is>
-          <t>dim_product: Hentet via join (SubLower[Subcategory]) → dim_product: Omdøbt (Subcategory → subcategory) → dim_product: Samlet (append) (Typer, Ukendt)</t>
+          <t>slv_subcategory: Navigation (subcategories (Sheet)) → slv_subcategory: Opdelt (CategorySubcategory → Subcategory (skilletegn "|")) → slv_subcategory: Transformeret ({"Subcategory", each Text.Proper(Text.Trim(_)), type text}) → dim_product: Hentet via join (SubLower[Subcategory]) → dim_product: Omdøbt (Subcategory → subcategory) → dim_product: Samlet (append) (Typer, Ukendt)</t>
         </is>
       </c>
       <c r="M36" s="5" t="inlineStr"/>
@@ -4055,7 +4251,11 @@
       </c>
       <c r="R36" s="4" t="inlineStr"/>
       <c r="S36" s="4" t="inlineStr"/>
-      <c r="T36" s="4" t="inlineStr"/>
+      <c r="T36" s="4" t="inlineStr">
+        <is>
+          <t>data/silver/Silver_Excel.xlsx › subcategories › CategorySubcategory (delen efter "|"); produkter matches via products › SubcategoryName</t>
+        </is>
+      </c>
       <c r="U36" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -4123,7 +4323,11 @@
       </c>
       <c r="R37" s="4" t="inlineStr"/>
       <c r="S37" s="4" t="inlineStr"/>
-      <c r="T37" s="4" t="inlineStr"/>
+      <c r="T37" s="4" t="inlineStr">
+        <is>
+          <t>data/silver/Silver_Excel.xlsx › products › UnitPrice</t>
+        </is>
+      </c>
       <c r="U37" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -4187,7 +4391,11 @@
       </c>
       <c r="R38" s="4" t="inlineStr"/>
       <c r="S38" s="4" t="inlineStr"/>
-      <c r="T38" s="4" t="inlineStr"/>
+      <c r="T38" s="4" t="inlineStr">
+        <is>
+          <t>data/silver/Silver_Excel.xlsx › products › PrimarySupplier</t>
+        </is>
+      </c>
       <c r="U38" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -4259,7 +4467,11 @@
       </c>
       <c r="R39" s="4" t="inlineStr"/>
       <c r="S39" s="4" t="inlineStr"/>
-      <c r="T39" s="4" t="inlineStr"/>
+      <c r="T39" s="4" t="inlineStr">
+        <is>
+          <t>Surrogatnøgle genereret i Power Query (fortløbende, -1 = Ukendt)</t>
+        </is>
+      </c>
       <c r="U39" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -4331,7 +4543,11 @@
           <t>Mulig PII - vurdér</t>
         </is>
       </c>
-      <c r="T40" s="4" t="inlineStr"/>
+      <c r="T40" s="4" t="inlineStr">
+        <is>
+          <t>data/silver/Silver_Excel.xlsx › cities › RegionName</t>
+        </is>
+      </c>
       <c r="U40" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -4403,7 +4619,11 @@
       </c>
       <c r="R41" s="4" t="inlineStr"/>
       <c r="S41" s="4" t="inlineStr"/>
-      <c r="T41" s="4" t="inlineStr"/>
+      <c r="T41" s="4" t="inlineStr">
+        <is>
+          <t>data/silver/Silver_Excel.xlsx › CAMPAIGN_LOG › Date</t>
+        </is>
+      </c>
       <c r="U41" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -4471,7 +4691,11 @@
       </c>
       <c r="R42" s="4" t="inlineStr"/>
       <c r="S42" s="4" t="inlineStr"/>
-      <c r="T42" s="4" t="inlineStr"/>
+      <c r="T42" s="4" t="inlineStr">
+        <is>
+          <t>Opslag af dim_campaign[campaign_key] (surrogatnøgle genereret i Power Query)</t>
+        </is>
+      </c>
       <c r="U42" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -4543,7 +4767,11 @@
       </c>
       <c r="R43" s="4" t="inlineStr"/>
       <c r="S43" s="4" t="inlineStr"/>
-      <c r="T43" s="4" t="inlineStr"/>
+      <c r="T43" s="4" t="inlineStr">
+        <is>
+          <t>data/silver/Silver_Excel.xlsx › CAMPAIGN_LOG › Impressions</t>
+        </is>
+      </c>
       <c r="U43" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -4615,7 +4843,11 @@
       </c>
       <c r="R44" s="4" t="inlineStr"/>
       <c r="S44" s="4" t="inlineStr"/>
-      <c r="T44" s="4" t="inlineStr"/>
+      <c r="T44" s="4" t="inlineStr">
+        <is>
+          <t>data/silver/Silver_Excel.xlsx › CAMPAIGN_LOG › Clicks</t>
+        </is>
+      </c>
       <c r="U44" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -4687,7 +4919,11 @@
       </c>
       <c r="R45" s="4" t="inlineStr"/>
       <c r="S45" s="4" t="inlineStr"/>
-      <c r="T45" s="4" t="inlineStr"/>
+      <c r="T45" s="4" t="inlineStr">
+        <is>
+          <t>data/silver/Silver_Excel.xlsx › CAMPAIGN_LOG › Spend</t>
+        </is>
+      </c>
       <c r="U45" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -4755,7 +4991,11 @@
       </c>
       <c r="R46" s="4" t="inlineStr"/>
       <c r="S46" s="4" t="inlineStr"/>
-      <c r="T46" s="4" t="inlineStr"/>
+      <c r="T46" s="4" t="inlineStr">
+        <is>
+          <t>data/silver/Silver_Excel.xlsx › inventory › kolonneoverskrifterne (yyyy-MM) efter unpivot, som første dag i måneden</t>
+        </is>
+      </c>
       <c r="U46" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -4823,7 +5063,11 @@
       </c>
       <c r="R47" s="4" t="inlineStr"/>
       <c r="S47" s="4" t="inlineStr"/>
-      <c r="T47" s="4" t="inlineStr"/>
+      <c r="T47" s="4" t="inlineStr">
+        <is>
+          <t>Opslag af dim_product[product_key] (surrogatnøgle genereret i Power Query)</t>
+        </is>
+      </c>
       <c r="U47" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -4871,7 +5115,7 @@
       <c r="I48" t="inlineStr"/>
       <c r="J48" t="inlineStr">
         <is>
-          <t>inventory (Sheet).StockQty</t>
+          <t>inventory (Sheet).(alle kolonner undtagen ProductName)</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -4881,7 +5125,7 @@
       </c>
       <c r="L48" s="5" t="inlineStr">
         <is>
-          <t>slv_inventory: Navigation (inventory (Sheet)) → fact_inventory: Omdøbt (StockQty → stock_qty)</t>
+          <t>slv_inventory: Navigation (inventory (Sheet)) → slv_inventory: Unpivot (StockQty = værdier fra alle kolonner undtagen ProductName) → fact_inventory: Omdøbt (StockQty → stock_qty)</t>
         </is>
       </c>
       <c r="M48" s="5" t="inlineStr"/>
@@ -4895,7 +5139,11 @@
       </c>
       <c r="R48" s="4" t="inlineStr"/>
       <c r="S48" s="4" t="inlineStr"/>
-      <c r="T48" s="4" t="inlineStr"/>
+      <c r="T48" s="4" t="inlineStr">
+        <is>
+          <t>data/silver/Silver_Excel.xlsx › inventory › værdierne i månedskolonnerne (unpivot, alle kolonner undtagen ProductName)</t>
+        </is>
+      </c>
       <c r="U48" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -4959,7 +5207,11 @@
       </c>
       <c r="R49" s="4" t="inlineStr"/>
       <c r="S49" s="4" t="inlineStr"/>
-      <c r="T49" s="4" t="inlineStr"/>
+      <c r="T49" s="4" t="inlineStr">
+        <is>
+          <t>data/silver/Silver_Excel.xlsx › order_line_items › LineID</t>
+        </is>
+      </c>
       <c r="U49" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -5023,7 +5275,11 @@
       </c>
       <c r="R50" s="4" t="inlineStr"/>
       <c r="S50" s="4" t="inlineStr"/>
-      <c r="T50" s="4" t="inlineStr"/>
+      <c r="T50" s="4" t="inlineStr">
+        <is>
+          <t>data/silver/Silver_Excel.xlsx › order_line_items › OrderID</t>
+        </is>
+      </c>
       <c r="U50" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -5095,7 +5351,11 @@
       </c>
       <c r="R51" s="4" t="inlineStr"/>
       <c r="S51" s="4" t="inlineStr"/>
-      <c r="T51" s="4" t="inlineStr"/>
+      <c r="T51" s="4" t="inlineStr">
+        <is>
+          <t>data/silver/Silver_Excel.xlsx › ORDERS_2025 + ORDERS_2026 › OrderDate (dato uden klokkeslæt)</t>
+        </is>
+      </c>
       <c r="U51" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -5163,7 +5423,11 @@
       </c>
       <c r="R52" s="4" t="inlineStr"/>
       <c r="S52" s="4" t="inlineStr"/>
-      <c r="T52" s="4" t="inlineStr"/>
+      <c r="T52" s="4" t="inlineStr">
+        <is>
+          <t>Opslag af dim_customer[customer_key] (surrogatnøgle genereret i Power Query)</t>
+        </is>
+      </c>
       <c r="U52" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -5231,7 +5495,11 @@
       </c>
       <c r="R53" s="4" t="inlineStr"/>
       <c r="S53" s="4" t="inlineStr"/>
-      <c r="T53" s="4" t="inlineStr"/>
+      <c r="T53" s="4" t="inlineStr">
+        <is>
+          <t>Opslag af dim_product[product_key] (surrogatnøgle genereret i Power Query)</t>
+        </is>
+      </c>
       <c r="U53" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -5299,7 +5567,11 @@
       </c>
       <c r="R54" s="4" t="inlineStr"/>
       <c r="S54" s="4" t="inlineStr"/>
-      <c r="T54" s="4" t="inlineStr"/>
+      <c r="T54" s="4" t="inlineStr">
+        <is>
+          <t>data/silver/Silver_Excel.xlsx › ORDERS_2025/ORDERS_2026 › OrderChannel, matchet mod dim_channel (ukendt → -1)</t>
+        </is>
+      </c>
       <c r="U54" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -5367,7 +5639,11 @@
       </c>
       <c r="R55" s="4" t="inlineStr"/>
       <c r="S55" s="4" t="inlineStr"/>
-      <c r="T55" s="4" t="inlineStr"/>
+      <c r="T55" s="4" t="inlineStr">
+        <is>
+          <t>Opslag af dim_region[region_key] (surrogatnøgle genereret i Power Query)</t>
+        </is>
+      </c>
       <c r="U55" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -5431,7 +5707,11 @@
       </c>
       <c r="R56" s="4" t="inlineStr"/>
       <c r="S56" s="4" t="inlineStr"/>
-      <c r="T56" s="4" t="inlineStr"/>
+      <c r="T56" s="4" t="inlineStr">
+        <is>
+          <t>data/silver/Silver_Excel.xlsx › ORDERS_2025 + ORDERS_2026 › Status (oversat til dansk)</t>
+        </is>
+      </c>
       <c r="U56" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -5495,7 +5775,11 @@
       </c>
       <c r="R57" s="4" t="inlineStr"/>
       <c r="S57" s="4" t="inlineStr"/>
-      <c r="T57" s="4" t="inlineStr"/>
+      <c r="T57" s="4" t="inlineStr">
+        <is>
+          <t>data/silver/Silver_Excel.xlsx › ORDERS_2025 + ORDERS_2026 › Priority (Express → Ekspres)</t>
+        </is>
+      </c>
       <c r="U57" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -5567,7 +5851,11 @@
       </c>
       <c r="R58" s="4" t="inlineStr"/>
       <c r="S58" s="4" t="inlineStr"/>
-      <c r="T58" s="4" t="inlineStr"/>
+      <c r="T58" s="4" t="inlineStr">
+        <is>
+          <t>data/silver/Silver_Excel.xlsx › order_line_items › Quantity</t>
+        </is>
+      </c>
       <c r="U58" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -5639,7 +5927,11 @@
       </c>
       <c r="R59" s="4" t="inlineStr"/>
       <c r="S59" s="4" t="inlineStr"/>
-      <c r="T59" s="4" t="inlineStr"/>
+      <c r="T59" s="4" t="inlineStr">
+        <is>
+          <t>data/silver/Silver_Excel.xlsx › order_line_items › UnitPrice</t>
+        </is>
+      </c>
       <c r="U59" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -5711,7 +6003,11 @@
       </c>
       <c r="R60" s="4" t="inlineStr"/>
       <c r="S60" s="4" t="inlineStr"/>
-      <c r="T60" s="4" t="inlineStr"/>
+      <c r="T60" s="4" t="inlineStr">
+        <is>
+          <t>data/silver/Silver_Excel.xlsx › order_line_items › DiscountPct</t>
+        </is>
+      </c>
       <c r="U60" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -5779,7 +6075,11 @@
       </c>
       <c r="R61" s="4" t="inlineStr"/>
       <c r="S61" s="4" t="inlineStr"/>
-      <c r="T61" s="4" t="inlineStr"/>
+      <c r="T61" s="4" t="inlineStr">
+        <is>
+          <t>Beregnet i Power Query: Quantity × UnitPrice fra data/silver/Silver_Excel.xlsx › order_line_items</t>
+        </is>
+      </c>
       <c r="U61" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -5847,7 +6147,11 @@
       </c>
       <c r="R62" s="4" t="inlineStr"/>
       <c r="S62" s="4" t="inlineStr"/>
-      <c r="T62" s="4" t="inlineStr"/>
+      <c r="T62" s="4" t="inlineStr">
+        <is>
+          <t>Beregnet i Power Query: gross_amount − net_amount</t>
+        </is>
+      </c>
       <c r="U62" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -5915,7 +6219,11 @@
       </c>
       <c r="R63" s="4" t="inlineStr"/>
       <c r="S63" s="4" t="inlineStr"/>
-      <c r="T63" s="4" t="inlineStr"/>
+      <c r="T63" s="4" t="inlineStr">
+        <is>
+          <t>Beregnet i Power Query: gross_amount × (1 − DiscountPct) fra data/silver/Silver_Excel.xlsx › order_line_items</t>
+        </is>
+      </c>
       <c r="U63" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -5983,7 +6291,11 @@
       </c>
       <c r="R64" s="4" t="inlineStr"/>
       <c r="S64" s="4" t="inlineStr"/>
-      <c r="T64" s="4" t="inlineStr"/>
+      <c r="T64" s="4" t="inlineStr">
+        <is>
+          <t>Beregnet i Power Query: Quantity × UnitCost fra data/silver/Silver_Excel.xlsx › order_line_items</t>
+        </is>
+      </c>
       <c r="U64" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -6051,7 +6363,11 @@
       </c>
       <c r="R65" s="4" t="inlineStr"/>
       <c r="S65" s="4" t="inlineStr"/>
-      <c r="T65" s="4" t="inlineStr"/>
+      <c r="T65" s="4" t="inlineStr">
+        <is>
+          <t>data/silver/Silver_Excel.xlsx › sales_targets › Period (yyyy-MM) som første dag i måneden</t>
+        </is>
+      </c>
       <c r="U65" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -6123,7 +6439,11 @@
       </c>
       <c r="R66" s="4" t="inlineStr"/>
       <c r="S66" s="4" t="inlineStr"/>
-      <c r="T66" s="4" t="inlineStr"/>
+      <c r="T66" s="4" t="inlineStr">
+        <is>
+          <t>data/silver/Silver_Excel.xlsx › sales_targets › TargetRevenue</t>
+        </is>
+      </c>
       <c r="U66" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -6199,7 +6519,11 @@
           <t>Mulig PII - vurdér</t>
         </is>
       </c>
-      <c r="T67" s="4" t="inlineStr"/>
+      <c r="T67" s="4" t="inlineStr">
+        <is>
+          <t>data/silver/Silver_Excel.xlsx › security › UserEmail (små bogstaver, trimmet)</t>
+        </is>
+      </c>
       <c r="U67" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>
@@ -6267,7 +6591,11 @@
       </c>
       <c r="R68" s="4" t="inlineStr"/>
       <c r="S68" s="4" t="inlineStr"/>
-      <c r="T68" s="4" t="inlineStr"/>
+      <c r="T68" s="4" t="inlineStr">
+        <is>
+          <t>data/silver/Silver_Excel.xlsx › security › Region</t>
+        </is>
+      </c>
       <c r="U68" s="4" t="inlineStr">
         <is>
           <t>Godkendt</t>

</xml_diff>